<commit_message>
Update analysis scripts, outputs, and models
</commit_message>
<xml_diff>
--- a/outputs/issues/cluster_topics_labeled.xlsx
+++ b/outputs/issues/cluster_topics_labeled.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +458,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>39</v>
+        <v>184</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -491,7 +491,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -557,21 +557,21 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -581,7 +581,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>36</v>
+        <v>172</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>761</v>
+        <v>54</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -656,21 +656,21 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>102</v>
+        <v>29</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -689,21 +689,21 @@
         <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -722,7 +722,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -755,21 +755,21 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -788,21 +788,21 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -821,21 +821,21 @@
         <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="n">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="n">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -920,21 +920,21 @@
         <v>14</v>
       </c>
       <c r="B16" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -953,21 +953,21 @@
         <v>15</v>
       </c>
       <c r="B17" t="n">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -986,21 +986,21 @@
         <v>16</v>
       </c>
       <c r="B18" t="n">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="n">
-        <v>30</v>
+        <v>111</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="n">
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="n">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1118,7 +1118,7 @@
         <v>20</v>
       </c>
       <c r="B22" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1151,21 +1151,21 @@
         <v>21</v>
       </c>
       <c r="B23" t="n">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -1184,21 +1184,21 @@
         <v>22</v>
       </c>
       <c r="B24" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1217,7 @@
         <v>23</v>
       </c>
       <c r="B25" t="n">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1250,31 +1250,31 @@
         <v>24</v>
       </c>
       <c r="B26" t="n">
-        <v>15</v>
+        <v>148</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Food Quality Issues</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Food Quality</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers raise concerns about inconsistent taste, poor preparation, or disappointing food quality.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Food was bland, poorly prepared, or did not meet expectations.</t>
         </is>
       </c>
     </row>
@@ -1283,31 +1283,31 @@
         <v>25</v>
       </c>
       <c r="B27" t="n">
-        <v>101</v>
+        <v>24</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Food Quality Issues</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Food Quality</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers raise concerns about inconsistent taste, poor preparation, or disappointing food quality.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Food was bland, poorly prepared, or did not meet expectations.</t>
         </is>
       </c>
     </row>
@@ -1316,21 +1316,21 @@
         <v>26</v>
       </c>
       <c r="B28" t="n">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -1349,31 +1349,31 @@
         <v>27</v>
       </c>
       <c r="B29" t="n">
-        <v>150</v>
+        <v>28</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Food Quality Issues</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Food Quality</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers raise concerns about inconsistent taste, poor preparation, or disappointing food quality.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Food was bland, poorly prepared, or did not meet expectations.</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1415,21 +1415,21 @@
         <v>29</v>
       </c>
       <c r="B31" t="n">
-        <v>221</v>
+        <v>20</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -1448,21 +1448,21 @@
         <v>30</v>
       </c>
       <c r="B32" t="n">
-        <v>62</v>
+        <v>180</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="n">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1514,7 +1514,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="n">
-        <v>307</v>
+        <v>59</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1547,7 +1547,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1580,21 +1580,21 @@
         <v>34</v>
       </c>
       <c r="B36" t="n">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
         <v>35</v>
       </c>
       <c r="B37" t="n">
-        <v>147</v>
+        <v>270</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1646,7 +1646,7 @@
         <v>36</v>
       </c>
       <c r="B38" t="n">
-        <v>15</v>
+        <v>141</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1679,31 +1679,31 @@
         <v>37</v>
       </c>
       <c r="B39" t="n">
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Food Quality Issues</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Food Quality</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Customers raise concerns about inconsistent taste, poor preparation, or disappointing food quality.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Food was bland, poorly prepared, or did not meet expectations.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1712,7 @@
         <v>38</v>
       </c>
       <c r="B40" t="n">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1745,7 +1745,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1778,7 +1778,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1811,21 +1811,21 @@
         <v>41</v>
       </c>
       <c r="B43" t="n">
-        <v>27</v>
+        <v>76</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -1844,21 +1844,21 @@
         <v>42</v>
       </c>
       <c r="B44" t="n">
-        <v>255</v>
+        <v>47</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1877,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="n">
-        <v>25</v>
+        <v>295</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1943,7 +1943,7 @@
         <v>45</v>
       </c>
       <c r="B47" t="n">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1976,31 +1976,31 @@
         <v>46</v>
       </c>
       <c r="B48" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Food Quality Issues</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Food Quality</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Customers raise concerns about inconsistent taste, poor preparation, or disappointing food quality.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Food was bland, poorly prepared, or did not meet expectations.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -2009,21 +2009,21 @@
         <v>47</v>
       </c>
       <c r="B49" t="n">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -2042,21 +2042,21 @@
         <v>48</v>
       </c>
       <c r="B50" t="n">
-        <v>29</v>
+        <v>487</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2075,7 @@
         <v>49</v>
       </c>
       <c r="B51" t="n">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -2108,21 +2108,21 @@
         <v>50</v>
       </c>
       <c r="B52" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -2141,21 +2141,21 @@
         <v>51</v>
       </c>
       <c r="B53" t="n">
-        <v>93</v>
+        <v>41</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -2174,7 +2174,7 @@
         <v>52</v>
       </c>
       <c r="B54" t="n">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -2207,31 +2207,31 @@
         <v>53</v>
       </c>
       <c r="B55" t="n">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Food Quality Issues</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Food Quality</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers raise concerns about inconsistent taste, poor preparation, or disappointing food quality.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Food was bland, poorly prepared, or did not meet expectations.</t>
         </is>
       </c>
     </row>
@@ -2240,7 +2240,7 @@
         <v>54</v>
       </c>
       <c r="B56" t="n">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
         <v>55</v>
       </c>
       <c r="B57" t="n">
-        <v>97</v>
+        <v>46</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -2306,7 +2306,7 @@
         <v>56</v>
       </c>
       <c r="B58" t="n">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -2339,21 +2339,21 @@
         <v>57</v>
       </c>
       <c r="B59" t="n">
-        <v>33</v>
+        <v>90</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Service Issues</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Service Efficiency</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
         </is>
       </c>
     </row>
@@ -2372,31 +2372,31 @@
         <v>58</v>
       </c>
       <c r="B60" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Food Quality Issues</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Food Quality</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers raise concerns about inconsistent taste, poor preparation, or disappointing food quality.</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Food was bland, poorly prepared, or did not meet expectations.</t>
         </is>
       </c>
     </row>
@@ -2405,21 +2405,21 @@
         <v>59</v>
       </c>
       <c r="B61" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Service Issues</t>
+          <t>Crowd and Wait Time</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Service Efficiency</t>
+          <t>Wait Time/Crowding</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
+          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
+          <t>Customers had to wait a long time and struggled with crowded seating.</t>
         </is>
       </c>
     </row>
@@ -2438,196 +2438,31 @@
         <v>60</v>
       </c>
       <c r="B62" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Crowd and Wait Time</t>
+          <t>Food Quality Issues</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Wait Time/Crowding</t>
+          <t>Food Quality</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
+          <t>Customers raise concerns about inconsistent taste, poor preparation, or disappointing food quality.</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="n">
-        <v>61</v>
-      </c>
-      <c r="B63" t="n">
-        <v>40</v>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Crowd and Wait Time</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Wait Time/Crowding</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="n">
-        <v>62</v>
-      </c>
-      <c r="B64" t="n">
-        <v>73</v>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Service Issues</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Service Efficiency</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Customers report slow, inattentive, or rude service that makes the restaurant experience frustrating.</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>Staff were slow, inattentive, or failed to handle requests properly.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="n">
-        <v>63</v>
-      </c>
-      <c r="B65" t="n">
-        <v>31</v>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Crowd and Wait Time</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Wait Time/Crowding</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="n">
-        <v>64</v>
-      </c>
-      <c r="B66" t="n">
-        <v>28</v>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Crowd and Wait Time</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Wait Time/Crowding</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="n">
-        <v>65</v>
-      </c>
-      <c r="B67" t="n">
-        <v>42</v>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Crowd and Wait Time</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Wait Time/Crowding</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Customers are frustrated by long waits and crowded conditions that make the dining experience uncomfortable.</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>Customers had to wait a long time and struggled with crowded seating.</t>
+          <t>Food was bland, poorly prepared, or did not meet expectations.</t>
         </is>
       </c>
     </row>

</xml_diff>